<commit_message>
feat(CR-040): username theo ten that, auto-suggest + doi ten tai khoan demo
- src/lib/username.ts: usernameBase (bo dau, ten + viet tat ho dem) +
  suggestUsername (hau to so khi trung) + unit tests
- /school/users: go ho ten -> tu de xuat email @<domain truong>, sua tay duoc
- bootstrap-school.mjs: can_bo.email trong -> tu sinh + dedupe, them --domain
- rename-demo-accounts.mjs: doi 88 tai khoan demo prod sang quy uoc moi
  (gvcn@demo.scn -> anhptl@nd.scn...), admin giu nguyen
- email.ts + cron parent-digest: block moi *.scn (parent contacts la @mail.scn,
  block @demo.scn cu khong con cover)
- template xlsx + seed + 20 file docs/QA cap nhat email moi; regen pptx/docx

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/handover/templates/khoi-tao-truong.xlsx
+++ b/docs/handover/templates/khoi-tao-truong.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="154">
   <si>
     <t>FILE MAU KHOI TAO TRUONG MOI - SO CHU NHIEM SO</t>
   </si>
@@ -107,6 +107,12 @@
     <t xml:space="preserve">  - Email la khoa dinh danh: can_bo/gvcn/phu_huynh/giao_vien TKB deu tham chieu bang email.</t>
   </si>
   <si>
+    <t xml:space="preserve">  - can_bo.email de trong -&gt; tu sinh &lt;ten&gt;&lt;viet-tat-ho-dem&gt;@&lt;domain&gt; (Le Duy Linh -&gt; linhld@...,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    trung thi linhld1...). Tham chieu cheo (gvcn_email...) dung email tu sinh do.</t>
+  </si>
+  <si>
     <t xml:space="preserve">  - mat_khau toi thieu 8 ky tu; de trong o phu_huynh = chi tao ho so, khong cap tai khoan.</t>
   </si>
   <si>
@@ -155,16 +161,16 @@
     <t>Toán, Vật lý, Hóa học, Sinh học, Tin học, Công nghệ</t>
   </si>
   <si>
-    <t>lananh.pt@truong.vn</t>
+    <t>anhptl@truong.vn</t>
   </si>
   <si>
     <t>Tổ Văn - Xã hội</t>
   </si>
   <si>
-    <t>Ngữ văn, Tiếng Anh, Lịch sử, Địa lý, GDCD</t>
-  </si>
-  <si>
-    <t>hung.nv@truong.vn</t>
+    <t>Ngữ văn, Tiếng Anh, Lịch sử và Địa lý, Giáo dục công dân</t>
+  </si>
+  <si>
+    <t>hungnv@truong.vn</t>
   </si>
   <si>
     <t>Tổ Thể chất - Nghệ thuật</t>
@@ -173,13 +179,13 @@
     <t>Thể dục, Âm nhạc, Mỹ thuật</t>
   </si>
   <si>
-    <t>binh.vt@truong.vn</t>
+    <t>binhvt@truong.vn</t>
   </si>
   <si>
     <t>ho_ten (*)</t>
   </si>
   <si>
-    <t>email (*)</t>
+    <t>email</t>
   </si>
   <si>
     <t>mat_khau (*)</t>
@@ -212,7 +218,7 @@
     <t>Nguyễn Văn Hải</t>
   </si>
   <si>
-    <t>hai.nv@truong.vn</t>
+    <t>hainv@truong.vn</t>
   </si>
   <si>
     <t>MatKhau@2026</t>
@@ -254,7 +260,7 @@
     <t>Trần Văn Minh</t>
   </si>
   <si>
-    <t>minh.tv@truong.vn</t>
+    <t>minhtv@truong.vn</t>
   </si>
   <si>
     <t>GV023</t>
@@ -269,7 +275,7 @@
     <t>Lê Minh Đức</t>
   </si>
   <si>
-    <t>duc.lm@truong.vn</t>
+    <t>duclm@truong.vn</t>
   </si>
   <si>
     <t>pht</t>
@@ -281,13 +287,13 @@
     <t>Cử nhân Sư phạm</t>
   </si>
   <si>
-    <t>GDCD</t>
+    <t>Giáo dục công dân</t>
   </si>
   <si>
     <t>Phạm Thu Trang</t>
   </si>
   <si>
-    <t>trang.pt@truong.vn</t>
+    <t>trangpt@truong.vn</t>
   </si>
   <si>
     <t>ke_toan</t>
@@ -408,9 +414,6 @@
   </si>
   <si>
     <t>dien_thoai</t>
-  </si>
-  <si>
-    <t>email</t>
   </si>
   <si>
     <t>ma_hs_con (*)</t>
@@ -875,7 +878,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1054,6 +1057,16 @@
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1074,35 +1087,35 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1123,46 +1136,46 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1191,206 +1204,206 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J2" t="s">
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" t="s">
+        <v>78</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
         <v>45</v>
       </c>
-      <c r="C3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="K3" t="s">
         <v>73</v>
-      </c>
-      <c r="E3" t="s">
-        <v>74</v>
-      </c>
-      <c r="F3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G3" t="s">
-        <v>69</v>
-      </c>
-      <c r="H3" t="s">
-        <v>76</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E4" t="s">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J5" t="s">
         <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J6" t="s">
         <v>1</v>
@@ -1401,72 +1414,72 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" t="s">
+        <v>98</v>
+      </c>
+      <c r="I7" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" t="s">
         <v>48</v>
       </c>
-      <c r="C7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F7" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" t="s">
-        <v>96</v>
-      </c>
-      <c r="I7" t="s">
-        <v>35</v>
-      </c>
-      <c r="J7" t="s">
-        <v>46</v>
-      </c>
       <c r="K7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" t="s">
+        <v>101</v>
+      </c>
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" t="s">
         <v>51</v>
       </c>
-      <c r="C8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F8" t="s">
-        <v>99</v>
-      </c>
-      <c r="G8" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" t="s">
-        <v>100</v>
-      </c>
-      <c r="I8" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" t="s">
-        <v>49</v>
-      </c>
       <c r="K8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1488,41 +1501,41 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B2">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B3">
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
         <v>1</v>
@@ -1530,16 +1543,16 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B4">
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1562,79 +1575,79 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F4" t="s">
         <v>1</v>
@@ -1642,19 +1655,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F5" t="s">
         <v>1</v>
@@ -1681,79 +1694,79 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F3" t="s">
         <v>138</v>
-      </c>
-      <c r="B3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E3" t="s">
-        <v>117</v>
-      </c>
-      <c r="F3" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F4" t="s">
         <v>1</v>
@@ -1779,27 +1792,27 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1808,18 +1821,18 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1828,18 +1841,18 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1848,18 +1861,18 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
         <v>151</v>
-      </c>
-      <c r="E4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B5">
         <v>2</v>
@@ -1868,13 +1881,13 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>